<commit_message>
docs: correct the plans matrix and add a competitor sheet
Four corrections from review: the departments limit was dropped on purpose, so it
comes out of the matrix — and the website still advertising it becomes a gap of
its own. The accounts limit goes back in, as a limit distinct from channels: two
WhatsApp numbers are one channel and two accounts. Conversations moves to the top
of the essentials, since it is what the price is built on. Customers and reports
split into two groups.

New sheet compares BEON and respond.io. Both price on monthly active contacts
rather than raw conversations, both meter broadcasts separately, and respond.io
sells extra seats and charges for overage instead of blocking. Neither has an
automation builder gap as wide as ours. Our own edge is Arabic dialects, Salla and
Zid, and a $19 entry against respond.io's $79.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGHUnSrtQwLX2BGbB3j6wk
</commit_message>
<xml_diff>
--- a/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
+++ b/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
@@ -11,6 +11,7 @@
     <sheet name="مصفوفة المزايا" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="توحيد المصادر" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="النواقص" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="مقارنة المنافسين" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,6 +90,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00CBD5E1"/>
       <sz val="11"/>
     </font>
@@ -102,12 +109,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00166534"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
       <sz val="9"/>
     </font>
     <font>
@@ -155,12 +156,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -195,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -245,17 +246,17 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -280,6 +281,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,82 +949,82 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>القنوات المتصلة</t>
+          <t>المحادثات شهرياً</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>limits.channels</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>قناتان</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>5 قنوات</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>كل القنوات</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>كل القنوات</t>
+          <t>limits.conversations</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>بلا حد</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>عدد الموظفين</t>
+          <t>القنوات المتصلة</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>limits.agents</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>20</v>
+          <t>limits.channels</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>قناتان</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>5 قنوات</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>كل القنوات</t>
+        </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>بلا حد</t>
+          <t>كل القنوات</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>المحادثات شهرياً</t>
+          <t>عدد الحسابات المربوطة</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>limits.conversations</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>500</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+          <t>limits.accounts — حقل ناقص في النظام</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>بلا حد</t>
         </is>
@@ -1023,26 +1033,24 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>جهات الاتصال</t>
+          <t>عدد الموظفين</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>limits.contacts</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>بلا حد</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+          <t>limits.agents</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>بلا حد</t>
         </is>
@@ -1051,26 +1059,26 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>الأقسام</t>
+          <t>جهات الاتصال</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>حدّ جديد — غير موجود في النظام</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
+          <t>limits.contacts</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>بلا حد</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>بلا حد</t>
         </is>
@@ -1102,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1192,32 +1200,32 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>القنوات المتصلة</t>
+          <t>المحادثات شهرياً</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>كم قناة تقدر تربطها بحسابك</t>
+          <t>سقف المحادثات التي يتعامل معها حسابك في الشهر — وعليه يقوم سعر الباقة</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>قناتان</t>
+          <t>500</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>5 قنوات</t>
+          <t>2,500</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>كل القنوات</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>كل القنوات</t>
+          <t>بلا حد</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -1239,32 +1247,32 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>عدد الموظفين</t>
+          <t>القنوات المتصلة</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>كم زميل يشتغل معك على نفس الحساب</t>
+          <t>نوع القناة: واتساب، إنستغرام، بريد… كم نوعاً تفتح لك الباقة</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>قناتان</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5 قنوات</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>كل القنوات</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>بلا حد</t>
+          <t>كل القنوات</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1286,27 +1294,27 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>المحادثات شهرياً</t>
+          <t>عدد الحسابات المربوطة</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>سقف المحادثات التي يتعامل معها حسابك في الشهر</t>
+          <t>كم حساباً فعلياً تربط — رقمَي واتساب مثلاً حسابان لا قناة واحدة</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2,500</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>10,000</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
@@ -1319,9 +1327,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>❌ غير منفّذ</t>
         </is>
       </c>
     </row>
@@ -1333,27 +1341,27 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>جهات الاتصال</t>
+          <t>عدد الموظفين</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>كم عميل تقدر تحفظ بياناته</t>
+          <t>كم زميل يشتغل معك على نفس الحساب</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>10,000</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>بلا حد</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
@@ -1380,27 +1388,27 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>الأقسام</t>
+          <t>جهات الاتصال</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>تقسيم الفريق لمجموعات وتوجيه المحادثات لكل قسم</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>كم عميل تقدر تحفظ بياناته</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>1,000</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>بلا حد</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
@@ -1435,32 +1443,32 @@
           <t>تطلب حدوداً تناسب حجمك وتتابع حالة طلبك حتى الاشتراك</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="20" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1489,32 +1497,32 @@
           <t>الرد على عملائك من رقم الواتساب الرسمي</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H13" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="20" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1536,22 +1544,22 @@
           <t>نافذة محادثة تحطها في موقعك ليكلمك الزائر مباشرة</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -1561,7 +1569,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr">
+      <c r="I14" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1583,32 +1591,32 @@
           <t>رسائل إنستغرام تصلك في نفس الصندوق</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G15" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="20" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1630,32 +1638,32 @@
           <t>رسائل صفحتك على فيسبوك</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G16" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="20" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1677,32 +1685,32 @@
           <t>محادثات تيليجرام</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G17" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H17" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="20" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1724,32 +1732,32 @@
           <t>Gmail و Outlook و Yahoo وأي بريد عبر SMTP</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G18" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1771,32 +1779,32 @@
           <t>الرسائل الخاصة على X</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G19" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H19" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="20" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1818,22 +1826,22 @@
           <t>يظهر لك طلب العميل وحالته وأنت ترد عليه</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -1843,7 +1851,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I20" s="20" t="inlineStr">
+      <c r="I20" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1865,22 +1873,22 @@
           <t>نفس الربط لمتاجر شوبيفاي وووكومرس</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -1890,7 +1898,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I21" s="20" t="inlineStr">
+      <c r="I21" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1919,32 +1927,32 @@
           <t>كل الرسائل من كل القنوات في مكان واحد، فلا تضيع محادثة</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G23" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H23" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="20" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H23" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -1966,32 +1974,32 @@
           <t>تكتب ملاحظة لزميلك داخل المحادثة لا يراها العميل</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="20" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2013,32 +2021,32 @@
           <t>تحفظ ردودك المتكررة وترسلها بضغطة</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G25" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="20" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2060,32 +2068,32 @@
           <t>تصنّف المحادثات بوسوم تبحث بها لاحقاً</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G26" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="20" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2107,32 +2115,32 @@
           <t>تسجّل وترسل رسالة صوتية من داخل المحادثة</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G27" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="20" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H27" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2154,32 +2162,32 @@
           <t>تصحّح رسالتك خلال 30 دقيقة من إرسالها</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G28" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H28" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="20" t="inlineStr">
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H28" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2208,22 +2216,22 @@
           <t>يرد على عملائك حتى خارج الدوام</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G30" s="18" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2255,22 +2263,22 @@
           <t>يفهم العربية بلهجاتها ويرد بنفس اللهجة</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G31" s="18" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F31" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2280,7 +2288,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I31" s="20" t="inlineStr">
+      <c r="I31" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2302,22 +2310,22 @@
           <t>ترفع منتجاتك وأسعارك وسياساتك فيرد منها لا بالتخمين</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F32" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G32" s="18" t="inlineStr">
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2327,7 +2335,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I32" s="20" t="inlineStr">
+      <c r="I32" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2349,22 +2357,22 @@
           <t>تحدّد أسلوبه: رسمي أو ودود أو مختصر، باسم علامتك</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G33" s="18" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2374,7 +2382,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I33" s="20" t="inlineStr">
+      <c r="I33" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2396,22 +2404,22 @@
           <t>يحوّل المحادثة للموظف المناسب ومعها ملخّص جاهز</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G34" s="18" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2421,7 +2429,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I34" s="20" t="inlineStr">
+      <c r="I34" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2443,32 +2451,32 @@
           <t>تحدّد مواضيع حسّاسة يمتنع عنها ويحوّلها للفريق</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E35" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F35" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G35" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H35" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="20" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H35" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2490,32 +2498,32 @@
           <t>كلمات مثل «موظف» أو «شكوى» تنقل المحادثة للفريق فوراً</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G36" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="20" t="inlineStr">
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H36" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2537,7 +2545,7 @@
           <t>عدد ردود المساعد المشمولة في باقتك</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D37" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2557,7 +2565,7 @@
           <t>مخصّص</t>
         </is>
       </c>
-      <c r="H37" s="19" t="inlineStr">
+      <c r="H37" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2584,32 +2592,32 @@
           <t>نبرة وقواعد مختلفة لكل قناة على حدة</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G38" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I38" s="20" t="inlineStr">
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H38" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2631,22 +2639,22 @@
           <t>يحوّل الرسالة الصوتية إلى نص تقرأه وتبحث فيه</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G39" s="18" t="inlineStr">
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2678,27 +2686,27 @@
           <t>يفهم الصورة أو ملف PDF الذي يرسله العميل</t>
         </is>
       </c>
-      <c r="D40" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G40" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H40" s="19" t="inlineStr">
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G40" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H40" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2725,27 +2733,27 @@
           <t>ينبّهك لما تكون نبرة العميل سلبية</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G41" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H41" s="19" t="inlineStr">
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G41" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H41" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2772,27 +2780,27 @@
           <t>يقترح رداً جاهزاً للموظف قبل أن يكتب</t>
         </is>
       </c>
-      <c r="D42" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F42" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G42" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H42" s="19" t="inlineStr">
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H42" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2819,27 +2827,27 @@
           <t>يتحسّن مع الوقت من أسلوب ردود موظفيك</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G43" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H43" s="19" t="inlineStr">
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G43" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H43" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2873,22 +2881,22 @@
           <t>ترسل عرضاً أو إعلاناً لقائمة عملائك على واتساب</t>
         </is>
       </c>
-      <c r="D45" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F45" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G45" s="18" t="inlineStr">
+      <c r="D45" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F45" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G45" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2898,7 +2906,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I45" s="20" t="inlineStr">
+      <c r="I45" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2920,22 +2928,22 @@
           <t>نفس الشيء عبر البريد</t>
         </is>
       </c>
-      <c r="D46" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F46" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G46" s="18" t="inlineStr">
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F46" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G46" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2945,7 +2953,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I46" s="20" t="inlineStr">
+      <c r="I46" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -2967,22 +2975,22 @@
           <t>قوالب رسائل تعدّلها بدل الكتابة من الصفر</t>
         </is>
       </c>
-      <c r="D47" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F47" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G47" s="18" t="inlineStr">
+      <c r="D47" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F47" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -2992,7 +3000,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I47" s="20" t="inlineStr">
+      <c r="I47" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3014,32 +3022,32 @@
           <t>ترسل الحملة لفئة محدّدة من عملائك لا للكل</t>
         </is>
       </c>
-      <c r="D48" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F48" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G48" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H48" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I48" s="20" t="inlineStr">
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G48" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H48" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3061,22 +3069,22 @@
           <t>كم وصلت وكم فُتحت وكم ردّوا</t>
         </is>
       </c>
-      <c r="D49" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G49" s="18" t="inlineStr">
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -3086,7 +3094,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I49" s="20" t="inlineStr">
+      <c r="I49" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3108,22 +3116,22 @@
           <t>تحدّد وقت الإرسال مسبقاً</t>
         </is>
       </c>
-      <c r="D50" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G50" s="18" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G50" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -3133,7 +3141,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I50" s="20" t="inlineStr">
+      <c r="I50" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3155,7 +3163,7 @@
           <t>سقف رسائل الحملات المشمولة — رسوم Meta منفصلة</t>
         </is>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3175,12 +3183,12 @@
           <t>مخصّص</t>
         </is>
       </c>
-      <c r="H51" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" s="21" t="inlineStr">
+      <c r="H51" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
         <is>
           <t>❌ غير منفّذ</t>
         </is>
@@ -3202,32 +3210,32 @@
           <t>يرسل على دفعات لحماية رقمك من الحظر</t>
         </is>
       </c>
-      <c r="D52" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G52" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H52" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I52" s="21" t="inlineStr">
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F52" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H52" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="17" t="inlineStr">
         <is>
           <t>❌ غير منفّذ</t>
         </is>
@@ -3256,22 +3264,22 @@
           <t>تحدّد ما يشوفه وما يعمله كل موظف</t>
         </is>
       </c>
-      <c r="D54" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F54" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G54" s="18" t="inlineStr">
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G54" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -3281,7 +3289,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I54" s="20" t="inlineStr">
+      <c r="I54" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3303,22 +3311,22 @@
           <t>رسالة تلقائية خارج أوقات عملكم</t>
         </is>
       </c>
-      <c r="D55" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F55" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G55" s="18" t="inlineStr">
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
         <is>
           <t>✔</t>
         </is>
@@ -3328,7 +3336,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I55" s="20" t="inlineStr">
+      <c r="I55" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3350,32 +3358,32 @@
           <t>الموظف يعلن حالته فلا تصله محادثات وهو مشغول</t>
         </is>
       </c>
-      <c r="D56" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G56" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H56" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I56" s="20" t="inlineStr">
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H56" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I56" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3397,27 +3405,27 @@
           <t>تحدّد خلال كم دقيقة يجب أن يصل أول رد</t>
         </is>
       </c>
-      <c r="D57" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G57" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F57" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H57" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3444,27 +3452,27 @@
           <t>محادثة فيها كلمة «فاتورة» تروح لقسم المحاسبة</t>
         </is>
       </c>
-      <c r="D58" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E58" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G58" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H58" s="19" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F58" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G58" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H58" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3491,27 +3499,27 @@
           <t>تشوف من فتح ومن ردّ ومن أغلق</t>
         </is>
       </c>
-      <c r="D59" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F59" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G59" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F59" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H59" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3538,32 +3546,32 @@
           <t>المحادثات تتوزّع على الفريق بالتساوي</t>
         </is>
       </c>
-      <c r="D60" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G60" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H60" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" s="21" t="inlineStr">
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H60" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I60" s="17" t="inlineStr">
         <is>
           <t>❌ غير منفّذ</t>
         </is>
@@ -3585,27 +3593,27 @@
           <t>طبقة حماية ثانية على حسابات فريقك</t>
         </is>
       </c>
-      <c r="D61" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F61" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G61" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H61" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3619,14 +3627,14 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -3639,32 +3647,32 @@
           <t>كل بيانات العميل وسجل محادثاته في مكان واحد</t>
         </is>
       </c>
-      <c r="D63" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G63" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" s="20" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H63" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3673,45 +3681,45 @@
     <row r="64" ht="26" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>قاعدة المعرفة</t>
+          <t>تصنيف العملاء</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>مقالات وأسئلة شائعة يستخدمها فريقك والمساعد</t>
-        </is>
-      </c>
-      <c r="D64" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E64" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G64" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H64" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I64" s="20" t="inlineStr">
+          <t>تقسم عملاءك لفئات تتعامل مع كل فئة بطريقة</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E64" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F64" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G64" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H64" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3720,45 +3728,45 @@
     <row r="65" ht="26" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>تصنيف العملاء</t>
+          <t>قاعدة المعرفة</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>تقسم عملاءك لفئات تتعامل مع كل فئة بطريقة</t>
-        </is>
-      </c>
-      <c r="D65" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F65" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G65" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H65" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I65" s="20" t="inlineStr">
+          <t>مقالات وأسئلة شائعة يستخدمها فريقك والمساعد</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E65" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F65" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G65" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H65" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3767,37 +3775,37 @@
     <row r="66" ht="26" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>تقارير الأداء</t>
+          <t>تقييمات العملاء</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>لوحة تشوف فيها حجم العمل وأداء الفريق</t>
-        </is>
-      </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>أساسية</t>
-        </is>
-      </c>
-      <c r="E66" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
-        </is>
-      </c>
-      <c r="F66" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
-        </is>
-      </c>
-      <c r="G66" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
+          <t>يقيّم العميل الخدمة بعد إغلاق المحادثة</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F66" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -3805,7 +3813,7 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I66" s="20" t="inlineStr">
+      <c r="I66" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3814,45 +3822,45 @@
     <row r="67" ht="26" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>متوسط زمن أول رد</t>
+          <t>الشكاوى والاقتراحات</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>كم يستنى عميلك قبل أول رد</t>
+          <t>صندوق منفصل للشكاوى تتابعه حتى الإغلاق</t>
         </is>
       </c>
       <c r="D67" s="18" t="inlineStr">
         <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E67" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F67" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G67" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H67" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I67" s="20" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F67" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G67" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H67" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -3861,139 +3869,99 @@
     <row r="68" ht="26" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>العملاء</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t>ساعات الذروة</t>
+          <t>سجل نشاط العميل</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>أي ساعات اليوم أكثر ضغطاً لتوزّع فريقك عليها</t>
-        </is>
-      </c>
-      <c r="D68" s="17" t="inlineStr">
+          <t>كل ما عمله العميل معك بالترتيب الزمني</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="E68" s="18" t="inlineStr">
         <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F68" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G68" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H68" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I68" s="20" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G68" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H68" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="26" customHeight="1">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>العملاء والتقارير</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>تقييمات العملاء</t>
-        </is>
-      </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>يقيّم العميل الخدمة بعد إغلاق المحادثة</t>
-        </is>
-      </c>
-      <c r="D69" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F69" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G69" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H69" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I69" s="20" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>التقارير</t>
         </is>
       </c>
     </row>
     <row r="70" ht="26" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>التقارير</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>الشكاوى والاقتراحات</t>
+          <t>تقارير الأداء</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>صندوق منفصل للشكاوى تتابعه حتى الإغلاق</t>
-        </is>
-      </c>
-      <c r="D70" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F70" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G70" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H70" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="20" t="inlineStr">
+          <t>لوحة تشوف فيها حجم العمل وأداء الفريق</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>أساسية</t>
+        </is>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="G70" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I70" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -4002,45 +3970,45 @@
     <row r="71" ht="26" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>التقارير</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>سجل نشاط العميل</t>
+          <t>متوسط زمن أول رد</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>كل ما عمله العميل معك بالترتيب الزمني</t>
-        </is>
-      </c>
-      <c r="D71" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G71" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H71" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" s="20" t="inlineStr">
+          <t>كم يستنى عميلك قبل أول رد</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E71" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F71" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G71" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H71" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
@@ -4049,148 +4017,148 @@
     <row r="72" ht="26" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>التقارير</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>تنبيه عند تأخّر الرد</t>
+          <t>ساعات الذروة</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>ينبّهك لما تتجاوز محادثة الوقت المسموح</t>
-        </is>
-      </c>
-      <c r="D72" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E72" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F72" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G72" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H72" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I72" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+          <t>أي ساعات اليوم أكثر ضغطاً لتوزّع فريقك عليها</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G72" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H72" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>العملاء والتقارير</t>
+          <t>التقارير</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
+          <t>تنبيه عند تأخّر الرد</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>ينبّهك لما تتجاوز محادثة الوقت المسموح</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G73" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H73" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>التقارير</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
           <t>تصدير التقارير</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C74" s="13" t="inlineStr">
         <is>
           <t>تنزّل تقاريرك ملف CSV</t>
         </is>
       </c>
-      <c r="D73" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E73" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F73" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G73" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H73" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I73" s="20" t="inlineStr">
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I74" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t>الربط والدعم</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>الربط والدعم</t>
-        </is>
-      </c>
-      <c r="B75" s="12" t="inlineStr">
-        <is>
-          <t>تكامل API</t>
-        </is>
-      </c>
-      <c r="C75" s="13" t="inlineStr">
-        <is>
-          <t>تربط Qhub بأنظمتك الأخرى</t>
-        </is>
-      </c>
-      <c r="D75" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E75" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F75" s="14" t="inlineStr">
-        <is>
-          <t>محدود</t>
-        </is>
-      </c>
-      <c r="G75" s="14" t="inlineStr">
-        <is>
-          <t>كامل</t>
-        </is>
-      </c>
-      <c r="H75" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I75" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -4202,32 +4170,32 @@
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>الدعم</t>
+          <t>تكامل API</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>كيف تتواصل معنا لما تحتاج مساعدة</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>بريد إلكتروني</t>
-        </is>
-      </c>
-      <c r="E76" s="14" t="inlineStr">
-        <is>
-          <t>أولوية</t>
+          <t>تربط Qhub بأنظمتك الأخرى</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
-          <t>أولوية</t>
+          <t>محدود</t>
         </is>
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
-          <t>مدير حساب</t>
+          <t>كامل</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
@@ -4249,95 +4217,143 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
+          <t>الدعم</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>كيف تتواصل معنا لما تحتاج مساعدة</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>بريد إلكتروني</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>أولوية</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>أولوية</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>مدير حساب</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I77" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>الربط والدعم</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
           <t>اتفاقية مستوى خدمة (SLA)</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
+      <c r="C78" s="13" t="inlineStr">
         <is>
           <t>التزام تعاقدي بزمن الرد ونسبة التشغيل</t>
         </is>
       </c>
-      <c r="D77" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F77" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="18" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I77" s="21" t="inlineStr">
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I78" s="17" t="inlineStr">
         <is>
           <t>❌ غير منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>المشمول في كل باقة</t>
         </is>
       </c>
-      <c r="C78" s="3">
-        <f>COUNTIF(H5:H77,"✔")&amp;" صفاً تظهر على الموقع"</f>
+      <c r="C79" s="3">
+        <f>COUNTIF(H5:H78,"✔")&amp;" صفاً تظهر على الموقع"</f>
         <v/>
       </c>
-      <c r="D78" s="3">
-        <f>COUNTIF(D5:D77,"✔")</f>
+      <c r="D79" s="3">
+        <f>COUNTIF(D5:D78,"✔")</f>
         <v/>
       </c>
-      <c r="E78" s="3">
-        <f>COUNTIF(E5:E77,"✔")</f>
+      <c r="E79" s="3">
+        <f>COUNTIF(E5:E78,"✔")</f>
         <v/>
       </c>
-      <c r="F78" s="3">
-        <f>COUNTIF(F5:F77,"✔")</f>
+      <c r="F79" s="3">
+        <f>COUNTIF(F5:F78,"✔")</f>
         <v/>
       </c>
-      <c r="G78" s="3">
-        <f>COUNTIF(G5:G77,"✔")</f>
+      <c r="G79" s="3">
+        <f>COUNTIF(G5:G78,"✔")</f>
         <v/>
       </c>
-      <c r="H78" s="3">
-        <f>COUNTIF(H5:H77,"✔")</f>
+      <c r="H79" s="3">
+        <f>COUNTIF(H5:H78,"✔")</f>
         <v/>
       </c>
-      <c r="I78" s="3">
-        <f>COUNTIF(I5:I77,"✅ منفّذ")&amp;" / "&amp;COUNTIF(I5:I77,"⚠️ جزئي")&amp;" / "&amp;COUNTIF(I5:I77,"❌ غير منفّذ")</f>
+      <c r="I79" s="3">
+        <f>COUNTIF(I5:I78,"✅ منفّذ")&amp;" / "&amp;COUNTIF(I5:I78,"⚠️ جزئي")&amp;" / "&amp;COUNTIF(I5:I78,"❌ غير منفّذ")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A75:I75"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A53:I53"/>
     <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A74:I74"/>
+    <mergeCell ref="A69:I69"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="A62:I62"/>
   </mergeCells>
@@ -4429,7 +4445,7 @@
           <t>المبتدئ</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>البداية</t>
         </is>
@@ -4461,7 +4477,7 @@
           <t>الاحترافي</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>الاحترافية</t>
         </is>
@@ -4493,7 +4509,7 @@
           <t>19 / 49 / 99 / 249</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>19 / 49 / 99 / 249</t>
         </is>
@@ -4525,7 +4541,7 @@
           <t>1 / 3 / 10 / بلا حد</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>2 / 5 / الكل / الكل</t>
         </is>
@@ -4557,7 +4573,7 @@
           <t>3 / 10 / 25 / بلا حد</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>2 / 7 / 20 / بلا حد</t>
         </is>
@@ -4589,7 +4605,7 @@
           <t>1,000 / 10,000 / 50,000 / بلا حد</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>500 / 2,500 / 10,000 / بلا حد</t>
         </is>
@@ -4621,7 +4637,7 @@
           <t>500 / بلا حد / بلا حد / بلا حد</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>1,000 / 10,000 / بلا حد / بلا حد</t>
         </is>
@@ -4635,7 +4651,7 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>الأقسام</t>
+          <t>حدّ الأقسام</t>
         </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
@@ -4650,24 +4666,24 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>الأقسام موجودة بلا حدّ للباقة</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>— / 3 / 10 / بلا حد</t>
+          <t>محذوف عمداً — قرار سابق</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>محذوف</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>إضافة limits.departments للنوع Plan — حدّ جديد بالكامل</t>
+          <t>إزالة صف «الأقسام» من جدول المقارنة في pricing.ts — الموقع لا يزال يعرض حدّاً أُلغي</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>عدد الحسابات</t>
+          <t>عدد الحسابات المربوطة</t>
         </is>
       </c>
       <c r="B13" s="22" t="inlineStr">
@@ -4682,17 +4698,17 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>لا وجود لهذا المفهوم</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>محذوف</t>
+          <t>لا وجود لهذا الحدّ</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>1 / 2 / 5 / بلا حد</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>لا شيء — البند شُطب، لا معنى له إلى جانب عدد الموظفين</t>
+          <t>إضافة limits.accounts للنوع Plan، وإضافة الصف لجدول الموقع. حدّ مستقل عن القنوات: رقمَا واتساب = قناة واحدة وحسابان.</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4733,7 @@
           <t>سعر معروض 249$ واشتراك ذاتي</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>بالتواصل مع المبيعات</t>
         </is>
@@ -4743,7 +4759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4834,17 +4850,17 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>حدّ الأقسام غير موجود أصلاً</t>
+          <t>عدد الحسابات المربوطة بلا حقل</t>
         </is>
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>الأقسام مبنية وتشتغل، لكن النوع Plan ما فيه limits.departments — فما في رقم يُقاس عليه.</t>
+          <t>حدّ مطلوب ومتّفق عليه، والنوع Plan ما فيه limits.accounts. القنوات في النظام صفوف مستقلة من نوع Channel، فربط رقمَي واتساب يُنشئ سجلّين تحت نوع واحد — أي أن التمييز بين «القناة» و«الحساب» قائم في البيانات وينقصه الحدّ فقط.</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>إضافة الحقل للنوع وللباقات الأربع قبل عرض الصف على الموقع.</t>
+          <t>إضافة limits.accounts للنوع وللباقات الأربع. أقرب حدّ للتنفيذ لأن البيانات جاهزة — يكفي عدّ سجلات Channel.</t>
         </is>
       </c>
     </row>
@@ -4854,17 +4870,17 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>تفريغ الرسائل الصوتية غير عامل</t>
+          <t>الموقع يعرض حدّاً محذوفاً</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>الواجهة كاملة، لكن transcribeAudio تُرجع نصاً ثابتاً، ولا شيء في التطبيق يشغّل المسار أصلاً.</t>
+          <t>جدول المقارنة في pricing.ts فيه صف «الأقسام: — / 3 / 10 / بلا حد»، وهذا الحدّ أُلغي عندنا عمداً.</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند — مفتاح المزوّد لا يوضع في المتصفح. البند معروض على الموقع اليوم.</t>
+          <t>حذف الصف من الموقع — نحن نَعِد بحدّ لم يعد موجوداً.</t>
         </is>
       </c>
     </row>
@@ -4874,17 +4890,17 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>المساعد الذكي كله يعتمد على دالة وهمية</t>
+          <t>تفريغ الرسائل الصوتية غير عامل</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>getAIResponse في utils/ai.ts تُرجع نصاً ثابتاً. كل صفوف «ردود تلقائية» و«اقتراح الرد» و«قراءة الصور» و«قياس الرضا» مفاتيح في الإعدادات بلا منطق خلفها.</t>
+          <t>الواجهة كاملة، لكن transcribeAudio تُرجع نصاً ثابتاً، ولا شيء في التطبيق يشغّل المسار أصلاً.</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند. الإعدادات والواجهات جاهزة بالكامل، ينقص الربط.</t>
+          <t>يحتاج باكند — مفتاح المزوّد لا يوضع في المتصفح. البند معروض على الموقع اليوم.</t>
         </is>
       </c>
     </row>
@@ -4894,17 +4910,17 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>أربع مزايا بلا أثر في الكود</t>
+          <t>المساعد الذكي كله يعتمد على دالة وهمية</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>توزيع تلقائي متوازن · إرسال تدريجي · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد.</t>
+          <t>getAIResponse في utils/ai.ts تُرجع نصاً ثابتاً. كل صفوف «ردود تلقائية» و«اقتراح الرد» و«قراءة الصور» و«قياس الرضا» مفاتيح في الإعدادات بلا منطق خلفها.</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>إما تُبنى أو تُشطب من العرض. اثنتان منها معروضتان على الموقع اليوم.</t>
+          <t>يحتاج باكند. الإعدادات والواجهات جاهزة بالكامل، ينقص الربط.</t>
         </is>
       </c>
     </row>
@@ -4914,17 +4930,17 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>بنود تُضبط ولا تُنفَّذ</t>
+          <t>أربع مزايا بلا أثر في الكود</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
+          <t>توزيع تلقائي متوازن · إرسال تدريجي · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد.</t>
         </is>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
+          <t>إما تُبنى أو تُشطب من العرض. اثنتان منها معروضتان على الموقع اليوم.</t>
         </is>
       </c>
     </row>
@@ -4934,17 +4950,17 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>بوابة الدفع غير منفّذة</t>
+          <t>بنود تُضبط ولا تُنفَّذ</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
+          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
+          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
         </is>
       </c>
     </row>
@@ -4954,17 +4970,17 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>الأمان في وضع عرض</t>
+          <t>بوابة الدفع غير منفّذة</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
+          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
         </is>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
+          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
         </is>
       </c>
     </row>
@@ -4974,17 +4990,17 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+          <t>الأمان في وضع عرض</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
         </is>
       </c>
     </row>
@@ -4994,15 +5010,35 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
+          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="56" customHeight="1">
+      <c r="A16" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
           <t>مزايا مبنية وغير معروضة</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>الرسائل الصوتية · تعديل الرسالة خلال 30 دقيقة · فهرسة دورات المحادثة · حالة متاح ومشغول · تصدير التقارير.</t>
         </is>
       </c>
-      <c r="D15" s="27" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>أُضيفت للمصفوفة. يستحق بعضها الظهور على الموقع — قرار تسويقي.</t>
         </is>
@@ -5015,4 +5051,483 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ما عند المنافسين وما ينقصنا</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>BEON من لقطة شاشة صفحة الباقات · respond.io من صفحة أسعارها ومراجعات 2026 (الدومين محجوب عن الوكيل، فالأرقام من مصادر ثانوية وتحتاج تأكيداً)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>BEON</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>respond.io</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>عندنا</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>التوصية</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>وحدة التسعير</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Conversations (MAC) — جهات اتصال نشطة شهرياً</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Monthly Active Contacts — نفس المفهوم، وهو المحور الأول للسعر</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>محادثات خام شهرياً</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>ندرس التحوّل لـ«جهة اتصال نشطة»: العميل الذي يراسلك 20 مرة يُحتسب مرة، وهو أعدل وأسهل تنبّؤاً — والمنافسان اتفقا عليه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>المحور الثاني للسعر</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Agents ثابت لكل باقة</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Users (مقاعد) — تُشترى إضافية بـ12–24$ للمقعد شهرياً</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>موظفون بعدد ثابت لا يُزاد</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>بيع مقعد إضافي دون ترقية الباقة — مصدر دخل مباشر ويمنع ترقية قسرية تُنفّر العميل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>تجاوز الحدّ</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>غير ظاهر</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>رسوم تجاوز: 12$ لكل 100 جهة على Growth و15$ على Advanced</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>لا حدّ يُطبَّق أصلاً</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>القرار الأهم: عند التجاوز نمنع أم نحاسب؟ respond.io تحاسب ولا توقف الخدمة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>صناديق الوارد / الحسابات</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Inboxes حدّ صريح: 4 / 10 / 10 / 5 / 1</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>تعدّد مساحات العمل على Advanced</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>الحدّ غائب — وهو «عدد الحسابات» المطلوب</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>يؤكّد قرارك: الحدّ ضروري وله سابقة عند المنافسين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>البثّ / الحملات</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Broadcasts حصّة مستقلة: 50 / 5k / 10k / 25k</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>البثّ لا يُفتح إلا من Growth فما فوق</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>الحملات مبنية بلا حصّة</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>إضافة حصّة رسائل حملات للباقة — عندنا الصف في المصفوفة بلا حقل وراءه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>حصص الذكاء الاصطناعي</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>حصّتان منفصلتان: AI Tokens و AI QA</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>أرصدة AI تكبر مع شريحة جهات الاتصال</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>رصيد واحد في الإعدادات غير مربوط بالباقة</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>ربط الرصيد بالباقة، وفصل «ردود» عن «تحليل» إن اختلفت كلفتهما.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>بناء الأتمتة</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Workflow Builds و Workflow Runs حصّتان</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Workflows محور رئيسي — ومعها HTTP requests على Advanced</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>لا يوجد بانٍ أتمتة إطلاقاً</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>أكبر فجوة وظيفية. عندنا توجيه بكلمة مفتاحية فقط، وهما عندهما محرّك كامل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>وكلاء AI</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>غير ظاهر</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>AI Agents — وكيل يدير المحادثة لا مجرّد ردّ آلي</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>مساعد يردّ ويحوّل</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>الفرق تسويقي بقدر ما هو تقني — «وكيل» أقوى من «ردّ تلقائي».</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>رصيد OTP و SMS</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>OTP Balance و SMS Balance حصّتان</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>SMS قناة مستقلة</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>فرصة دخل إضافي، ومطلوبة لأي تحقّق برقم الجوال.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>باقة مجانية دائمة</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Free forever — 50 محادثة و1 موظف و4 صناديق</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>تجربة 7 أيام فقط</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>تجربة يفتحها الأدمن يدوياً 14 يوماً</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>باقة مجانية دائمة أقوى قمع استحواذ من تجربة مؤقتة — قرار تجاري.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>باقات مخصّصة بالاسم</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>باقة باسم العميل: «Adel Sedik English Academy»</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Enterprise بترتيب مخصّص</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>مسار طلب حدود مخصّصة مبني بالكامل</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>نحن جاهزون هنا — ينقص فقط أن يُنشئ الأدمن باقة خاصة بعد الموافقة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>باقات حسب المجال</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>نسخ E-Commerce من كل باقة بحدود مختلفة</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>غير ظاهر</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>باقة واحدة للجميع</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>يستحق الدراسة: عندنا سلة وزد وشوبيفاي — باقة تجارة إلكترونية منطقية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>تسجيل دخول موحّد SSO</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>غير ظاهر</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>SSO على Advanced</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>مذكور في مزايا المؤسسات وغير مبني</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>مطلب مؤسسي متكرّر — يبقى حبراً على ورق حتى يُبنى.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>تطبيق جوال</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>غير ظاهر</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>تطبيق على كل الباقات بما فيها Starter</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>غير موجود</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>معروض في ملفك على ثلاث باقات ولا أثر له — إما يُبنى أو يُشطب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>ما نتفوّق به</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>اللهجات العربية · سلة وزد · واجهة عربية أصلية · أسعار أقل بكثير (19$ مقابل 79$)</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>هذه نقاط البيع. respond.io تبدأ من 79$ ونحن من 19$ — الفجوة السعرية وحدها رسالة تسويقية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>أسعارهم للمقارنة — BEON: من 1,199 ج.م إلى 12,399 ج.م شهرياً · respond.io: Starter 79$ · Growth 159$ · Advanced 279–349$ · نحن: 19$ إلى 249$</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A21:E21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: enterprise reads "on request", not $249
The 249 is real in both codebases, but contactOnly hides it on the website and
shows "on request" instead, so no customer has ever seen it. Printing it as the
enterprise price in the matrix was wrong.

Tracing it surfaced a genuine mismatch: the website treats enterprise as a
sales-led plan while the dashboard sells it self-serve, price on screen and a
checkout that completes. That contradicts the custom-limits request flow, and is
now recorded as a gap.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGHUnSrtQwLX2BGbB3j6wk
</commit_message>
<xml_diff>
--- a/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
+++ b/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
@@ -907,8 +907,10 @@
       <c r="E12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="F12" s="8" t="n">
-        <v>249</v>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>بالتواصل</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -934,9 +936,10 @@
         <f>E12*12*0.8</f>
         <v/>
       </c>
-      <c r="F13" s="8">
-        <f>F12*12*0.8</f>
-        <v/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>بالتواصل</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -4496,27 +4499,27 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
+          <t>19 / 49 / 99 — والمؤسسات «بالطلب»</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>#REF! — صيغ مكسورة</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
           <t>19 / 49 / 99 / 249</t>
         </is>
       </c>
-      <c r="C7" s="22" t="inlineStr">
-        <is>
-          <t>#REF! — صيغ مكسورة</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>19 / 49 / 99 / 249</t>
-        </is>
-      </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>19 / 49 / 99 / 249</t>
+          <t>19 / 49 / 99 / بالتواصل</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>لا شيء — الموقع والنظام متطابقان</t>
+          <t>الثلاث الأولى متطابقة. أما 249 فرقم قائم في الكود في الملفين ولا يراه أي عميل: contactOnly على الموقع يخفيه ويعرض «بالطلب». يُحذف من النظام أو يُحوَّل لسعر أساس داخلي يبني عليه فريق المبيعات.</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4723,7 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>بالتواصل — السعر يُتّفق عليه</t>
+          <t>contactOnly — تعرض «بالطلب» ولا تعرض رقماً</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
@@ -4730,7 +4733,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>سعر معروض 249$ واشتراك ذاتي</t>
+          <t>تُعامَل كباقة عادية: 249$ ظاهرة في /subscribe وزر اشتراك ذاتي</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
@@ -4740,7 +4743,7 @@
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>قرار تجاري: يُعرض السعر أم يبقى «تواصل معنا»؟</t>
+          <t>خلل فعلي: الموقع يقول «تواصل معنا» واللوحة تعرض السعر وتتيح الشراء المباشر. توحيد السلوك — لا اشتراك ذاتي على المؤسسات.</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4870,17 +4873,17 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>الموقع يعرض حدّاً محذوفاً</t>
+          <t>المؤسسات تُباع ذاتياً رغم أنها «بالطلب»</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>جدول المقارنة في pricing.ts فيه صف «الأقسام: — / 3 / 10 / بلا حد»، وهذا الحدّ أُلغي عندنا عمداً.</t>
+          <t>الموقع يخفي سعرها ويعرض «بالطلب» (contactOnly). اللوحة تعاملها كباقة عادية: 249$ ظاهرة في /subscribe مع زر اشتراك مباشر — تحققت من ذلك بفتح المسار، ويصل فعلاً لشاشة «إتمام الدفع».</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>حذف الصف من الموقع — نحن نَعِد بحدّ لم يعد موجوداً.</t>
+          <t>يناقض مسار طلب الحدود المخصّصة الذي بنيناه. المفروض لا اشتراك ذاتي على المؤسسات — الزر يقود للنموذج لا للدفع.</t>
         </is>
       </c>
     </row>
@@ -4890,17 +4893,17 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>تفريغ الرسائل الصوتية غير عامل</t>
+          <t>الموقع يعرض حدّاً محذوفاً</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>الواجهة كاملة، لكن transcribeAudio تُرجع نصاً ثابتاً، ولا شيء في التطبيق يشغّل المسار أصلاً.</t>
+          <t>جدول المقارنة في pricing.ts فيه صف «الأقسام: — / 3 / 10 / بلا حد»، وهذا الحدّ أُلغي عندنا عمداً.</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند — مفتاح المزوّد لا يوضع في المتصفح. البند معروض على الموقع اليوم.</t>
+          <t>حذف الصف من الموقع — نحن نَعِد بحدّ لم يعد موجوداً.</t>
         </is>
       </c>
     </row>
@@ -4910,17 +4913,17 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>المساعد الذكي كله يعتمد على دالة وهمية</t>
+          <t>تفريغ الرسائل الصوتية غير عامل</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>getAIResponse في utils/ai.ts تُرجع نصاً ثابتاً. كل صفوف «ردود تلقائية» و«اقتراح الرد» و«قراءة الصور» و«قياس الرضا» مفاتيح في الإعدادات بلا منطق خلفها.</t>
+          <t>الواجهة كاملة، لكن transcribeAudio تُرجع نصاً ثابتاً، ولا شيء في التطبيق يشغّل المسار أصلاً.</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند. الإعدادات والواجهات جاهزة بالكامل، ينقص الربط.</t>
+          <t>يحتاج باكند — مفتاح المزوّد لا يوضع في المتصفح. البند معروض على الموقع اليوم.</t>
         </is>
       </c>
     </row>
@@ -4930,17 +4933,17 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>أربع مزايا بلا أثر في الكود</t>
+          <t>المساعد الذكي كله يعتمد على دالة وهمية</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>توزيع تلقائي متوازن · إرسال تدريجي · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد.</t>
+          <t>getAIResponse في utils/ai.ts تُرجع نصاً ثابتاً. كل صفوف «ردود تلقائية» و«اقتراح الرد» و«قراءة الصور» و«قياس الرضا» مفاتيح في الإعدادات بلا منطق خلفها.</t>
         </is>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>إما تُبنى أو تُشطب من العرض. اثنتان منها معروضتان على الموقع اليوم.</t>
+          <t>يحتاج باكند. الإعدادات والواجهات جاهزة بالكامل، ينقص الربط.</t>
         </is>
       </c>
     </row>
@@ -4950,17 +4953,17 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>بنود تُضبط ولا تُنفَّذ</t>
+          <t>أربع مزايا بلا أثر في الكود</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
+          <t>توزيع تلقائي متوازن · إرسال تدريجي · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد.</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
+          <t>إما تُبنى أو تُشطب من العرض. اثنتان منها معروضتان على الموقع اليوم.</t>
         </is>
       </c>
     </row>
@@ -4970,17 +4973,17 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>بوابة الدفع غير منفّذة</t>
+          <t>بنود تُضبط ولا تُنفَّذ</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
+          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
         </is>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
+          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
         </is>
       </c>
     </row>
@@ -4990,17 +4993,17 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>الأمان في وضع عرض</t>
+          <t>بوابة الدفع غير منفّذة</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
+          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
+          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
         </is>
       </c>
     </row>
@@ -5010,17 +5013,17 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+          <t>الأمان في وضع عرض</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
         </is>
       </c>
     </row>
@@ -5030,15 +5033,35 @@
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
+          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
           <t>مزايا مبنية وغير معروضة</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>الرسائل الصوتية · تعديل الرسالة خلال 30 دقيقة · فهرسة دورات المحادثة · حالة متاح ومشغول · تصدير التقارير.</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>أُضيفت للمصفوفة. يستحق بعضها الظهور على الموقع — قرار تسويقي.</t>
         </is>

</xml_diff>

<commit_message>
docs: gradual campaign sending is built, not missing
My earlier search looked for "throttle", "gradual" and "batchSize" and found
nothing, so I marked the row as absent. It is named minDelay/maxDelay: four speed
presets from 5-15s to 60-180s, a risk indicator, an estimated campaign duration,
and per-template defaults. The search failed, the feature did not.

It is still partial rather than done, for a different reason: the Campaign type
carries no delay fields, so the setting is discarded when the campaign is saved.
Two fields away from complete.

Re-checked the other two absences while here. Balanced auto-distribution really
has no implementation — and a knowledge-base article tells customers it runs on
round robin, which is worth correcting on its own.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGHUnSrtQwLX2BGbB3j6wk
</commit_message>
<xml_diff>
--- a/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
+++ b/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
@@ -3210,7 +3210,7 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>يرسل على دفعات لحماية رقمك من الحظر</t>
+          <t>فترة بين كل رسالة وأخرى لحماية رقمك من الحظر</t>
         </is>
       </c>
       <c r="D52" s="18" t="inlineStr">
@@ -3233,14 +3233,14 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H52" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I52" s="17" t="inlineStr">
-        <is>
-          <t>❌ غير منفّذ</t>
+      <c r="H52" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I52" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4953,17 +4953,17 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>أربع مزايا بلا أثر في الكود</t>
+          <t>الإرسال التدريجي يُضبط ثم يُرمى</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>توزيع تلقائي متوازن · إرسال تدريجي · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد.</t>
+          <t>الواجهة مبنية بالكامل: أربع سرعات جاهزة (سريع 5-15ث · معتدل 15-45ث · حذر 30-90ث · آمن جداً 60-180ث)، ومؤشّر خطر، وتقدير لمدة الحملة، والقوالب تحمل سرعتها الافتراضية. لكن النوع Campaign ما فيه minDelay ولا maxDelay — الإعداد يعيش في نموذج الإنشاء ويضيع عند الحفظ.</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>إما تُبنى أو تُشطب من العرض. اثنتان منها معروضتان على الموقع اليوم.</t>
+          <t>أقرب بند للإنجاز في الملف كله: حقلان على النوع وحفظهما. الشغل الصعب (الواجهة والسرعات والمؤشّر) خلصان.</t>
         </is>
       </c>
     </row>
@@ -4973,17 +4973,17 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>بنود تُضبط ولا تُنفَّذ</t>
+          <t>ثلاث مزايا بلا أثر في الكود</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
+          <t>توزيع تلقائي متوازن · سقف رسائل الحملات · اتفاقية SLA. ولا واحدة منها لها سطر واحد. والأسوأ: مقال في قاعدة المعرفة يشرح للعميل أن التوزيع يتم «بنظام Round Robin» — وهو غير مبني.</t>
         </is>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
+          <t>إما تُبنى أو تُشطب. وعلى الأقل يُصحَّح مقال قاعدة المعرفة فوراً.</t>
         </is>
       </c>
     </row>
@@ -4993,17 +4993,17 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>بوابة الدفع غير منفّذة</t>
+          <t>بنود تُضبط ولا تُنفَّذ</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
+          <t>هدف زمن الاستجابة يُحفظ على القسم ولا تنبيه يُطلَق · كلمات التوجيه routingKeywords تُحفظ ولا كود يقرأها · سجلّ الإجراءات على مستوى المحادثة لا الموظف.</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
+          <t>ثلاثة بنود قريبة الإنجاز — الحقول موجودة، ينقص المنطق.</t>
         </is>
       </c>
     </row>
@@ -5013,17 +5013,17 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>الأمان في وضع عرض</t>
+          <t>بوابة الدفع غير منفّذة</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
+          <t>إعدادات Paymob ومفاتيحها موجودة، لكن زر «الانتقال للدفع» يصل لشاشة الدفع ولا يُحصّل شيئاً.</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
+          <t>يحتاج باكند. لا يظهر في المصفوفة لأنه واحد في كل الباقات.</t>
         </is>
       </c>
     </row>
@@ -5033,17 +5033,17 @@
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
-          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+          <t>الأمان في وضع عرض</t>
         </is>
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+          <t>التحقق بخطوتين يعمل في المتصفح بسرّ مشترك · رمز OTP يظهر في لافتة على الشاشة · دخول Google و Apple شاشة محاكاة بلا OAuth.</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+          <t>لا يُطرح للعملاء قبل الباكند. التحقق بخطوتين وحده مذكور في المصفوفة لأنه يختلف بين الباقات.</t>
         </is>
       </c>
     </row>
@@ -5053,15 +5053,35 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
+          <t>التجربة المجانية: 7 أيام أم 14؟</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>صفحة الأسعار تَعِد بـ«7 أيام مجاناً دون بطاقة». النظام يعرف الحالة التجريبية (ClientStatus «trial» و trialEndsAt)، لكن الأدمن وحده يفتحها يدوياً من شاشة العملاء — و**بمدة 14 يوماً** لا 7. التسجيل الذاتي لا ينشئ تجربة إطلاقاً، ولا شيء ينهيها عند انقضائها.</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>ثلاثة قرارات: توحيد المدة (7 أم 14)، وبدء التجربة تلقائياً عند التسجيل، وما الذي يحدث عند انتهائها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
           <t>مزايا مبنية وغير معروضة</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>الرسائل الصوتية · تعديل الرسالة خلال 30 دقيقة · فهرسة دورات المحادثة · حالة متاح ومشغول · تصدير التقارير.</t>
         </is>
       </c>
-      <c r="D17" s="27" t="inlineStr">
+      <c r="D18" s="27" t="inlineStr">
         <is>
           <t>أُضيفت للمصفوفة. يستحق بعضها الظهور على الموقع — قرار تسويقي.</t>
         </is>

</xml_diff>

<commit_message>
docs: the employee mobile app exists — it is a third repo
Marked absent because the audit read the dashboard and the website repos and the
app lives in neither. It is built and deployed at qhub-employee: conversations,
handover, voice messages, available/busy, tags, notifications, knowledge base,
internal notes.

So it moves from the gaps into the inbox group, and in the competitor sheet it
turns from a hole into an advantage we fail to advertise — respond.io sells its
app on every plan including the cheapest, and our pricing page never mentions ours.

Added a note on the audit's own scope, since this is the second finding that was
simply out of reach: any further repo may hold more of what this file calls
unimplemented.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGHUnSrtQwLX2BGbB3j6wk
</commit_message>
<xml_diff>
--- a/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
+++ b/docs/Qhub - مصفوفة الباقات والمزايا.xlsx
@@ -1113,7 +1113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2196,57 +2196,57 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>صندوق الوارد</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>تطبيق الموظفين على الجوال</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>فريقك يرد من جواله: المحادثات والتحويل والرسائل الصوتية وحالة متاح/مشغول</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I29" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>المساعد الذكي</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>المساعد الذكي</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>ردود تلقائية على مدار الساعة</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>يرد على عملائك حتى خارج الدوام</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F30" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G30" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I30" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -2258,12 +2258,12 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>يفهم اللغات واللهجات</t>
+          <t>ردود تلقائية على مدار الساعة</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>يفهم العربية بلهجاتها ويرد بنفس اللهجة</t>
+          <t>يرد على عملائك حتى خارج الدوام</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -2291,9 +2291,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -2305,12 +2305,12 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>قاعدة معرفة مخصّصة</t>
+          <t>يفهم اللغات واللهجات</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>ترفع منتجاتك وأسعارك وسياساتك فيرد منها لا بالتخمين</t>
+          <t>يفهم العربية بلهجاتها ويرد بنفس اللهجة</t>
         </is>
       </c>
       <c r="D32" s="18" t="inlineStr">
@@ -2352,12 +2352,12 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>أسلوب الرد</t>
+          <t>قاعدة معرفة مخصّصة</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>تحدّد أسلوبه: رسمي أو ودود أو مختصر، باسم علامتك</t>
+          <t>ترفع منتجاتك وأسعارك وسياساتك فيرد منها لا بالتخمين</t>
         </is>
       </c>
       <c r="D33" s="18" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>تحويل للموظف عند الحاجة</t>
+          <t>أسلوب الرد</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>يحوّل المحادثة للموظف المناسب ومعها ملخّص جاهز</t>
+          <t>تحدّد أسلوبه: رسمي أو ودود أو مختصر، باسم علامتك</t>
         </is>
       </c>
       <c r="D34" s="18" t="inlineStr">
@@ -2446,12 +2446,12 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>مواضيع لا يتكلم فيها</t>
+          <t>تحويل للموظف عند الحاجة</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>تحدّد مواضيع حسّاسة يمتنع عنها ويحوّلها للفريق</t>
+          <t>يحوّل المحادثة للموظف المناسب ومعها ملخّص جاهز</t>
         </is>
       </c>
       <c r="D35" s="18" t="inlineStr">
@@ -2474,9 +2474,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H35" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I35" s="21" t="inlineStr">
@@ -2493,12 +2493,12 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>تحويل فوري بكلمة</t>
+          <t>مواضيع لا يتكلم فيها</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>كلمات مثل «موظف» أو «شكوى» تنقل المحادثة للفريق فوراً</t>
+          <t>تحدّد مواضيع حسّاسة يمتنع عنها ويحوّلها للفريق</t>
         </is>
       </c>
       <c r="D36" s="18" t="inlineStr">
@@ -2540,12 +2540,12 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>رصيد الردود الشهري</t>
+          <t>تحويل فوري بكلمة</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>عدد ردود المساعد المشمولة في باقتك</t>
+          <t>كلمات مثل «موظف» أو «شكوى» تنقل المحادثة للفريق فوراً</t>
         </is>
       </c>
       <c r="D37" s="18" t="inlineStr">
@@ -2553,19 +2553,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="F37" s="14" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>مخصّص</t>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="H37" s="20" t="inlineStr">
@@ -2573,9 +2573,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I37" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="I37" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -2587,12 +2587,12 @@
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>إعدادات مستقلة لكل قناة</t>
+          <t>رصيد الردود الشهري</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>نبرة وقواعد مختلفة لكل قناة على حدة</t>
+          <t>عدد ردود المساعد المشمولة في باقتك</t>
         </is>
       </c>
       <c r="D38" s="18" t="inlineStr">
@@ -2600,19 +2600,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>مخصّص</t>
         </is>
       </c>
       <c r="H38" s="20" t="inlineStr">
@@ -2620,9 +2620,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I38" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2634,12 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>تفريغ الرسائل الصوتية</t>
+          <t>إعدادات مستقلة لكل قناة</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>يحوّل الرسالة الصوتية إلى نص تقرأه وتبحث فيه</t>
+          <t>نبرة وقواعد مختلفة لكل قناة على حدة</t>
         </is>
       </c>
       <c r="D39" s="18" t="inlineStr">
@@ -2662,14 +2662,14 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H39" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I39" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="H39" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -2681,12 +2681,12 @@
       </c>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>قراءة الصور والملفات</t>
+          <t>تفريغ الرسائل الصوتية</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>يفهم الصورة أو ملف PDF الذي يرسله العميل</t>
+          <t>يحوّل الرسالة الصوتية إلى نص تقرأه وتبحث فيه</t>
         </is>
       </c>
       <c r="D40" s="18" t="inlineStr">
@@ -2709,9 +2709,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H40" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I40" s="16" t="inlineStr">
@@ -2728,12 +2728,12 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>قياس رضا العميل أثناء المحادثة</t>
+          <t>قراءة الصور والملفات</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>ينبّهك لما تكون نبرة العميل سلبية</t>
+          <t>يفهم الصورة أو ملف PDF الذي يرسله العميل</t>
         </is>
       </c>
       <c r="D41" s="18" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>اقتراح الرد على الموظف</t>
+          <t>قياس رضا العميل أثناء المحادثة</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>يقترح رداً جاهزاً للموظف قبل أن يكتب</t>
+          <t>ينبّهك لما تكون نبرة العميل سلبية</t>
         </is>
       </c>
       <c r="D42" s="18" t="inlineStr">
@@ -2788,9 +2788,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F42" s="19" t="inlineStr">
@@ -2822,96 +2822,96 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
+          <t>اقتراح الرد على الموظف</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>يقترح رداً جاهزاً للموظف قبل أن يكتب</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G43" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H43" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>المساعد الذكي</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
           <t>يتعلّم من ردود فريقك</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>يتحسّن مع الوقت من أسلوب ردود موظفيك</t>
         </is>
       </c>
-      <c r="D43" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G43" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H43" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" s="16" t="inlineStr">
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H44" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
         <is>
           <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>التسويق والحملات</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>التسويق والحملات</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>حملات واتساب</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>ترسل عرضاً أو إعلاناً لقائمة عملائك على واتساب</t>
-        </is>
-      </c>
-      <c r="D45" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F45" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G45" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H45" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I45" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -2923,12 +2923,12 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>حملات بريد إلكتروني</t>
+          <t>حملات واتساب</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>نفس الشيء عبر البريد</t>
+          <t>ترسل عرضاً أو إعلاناً لقائمة عملائك على واتساب</t>
         </is>
       </c>
       <c r="D46" s="18" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>قوالب جاهزة</t>
+          <t>حملات بريد إلكتروني</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>قوالب رسائل تعدّلها بدل الكتابة من الصفر</t>
+          <t>نفس الشيء عبر البريد</t>
         </is>
       </c>
       <c r="D47" s="18" t="inlineStr">
@@ -3017,12 +3017,12 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>استهداف بالوسوم</t>
+          <t>قوالب جاهزة</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>ترسل الحملة لفئة محدّدة من عملائك لا للكل</t>
+          <t>قوالب رسائل تعدّلها بدل الكتابة من الصفر</t>
         </is>
       </c>
       <c r="D48" s="18" t="inlineStr">
@@ -3045,9 +3045,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H48" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I48" s="21" t="inlineStr">
@@ -3064,12 +3064,12 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>تقارير الحملات</t>
+          <t>استهداف بالوسوم</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>كم وصلت وكم فُتحت وكم ردّوا</t>
+          <t>ترسل الحملة لفئة محدّدة من عملائك لا للكل</t>
         </is>
       </c>
       <c r="D49" s="18" t="inlineStr">
@@ -3092,9 +3092,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H49" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
+      <c r="H49" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I49" s="21" t="inlineStr">
@@ -3111,12 +3111,12 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>جدولة الإرسال</t>
+          <t>تقارير الحملات</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>تحدّد وقت الإرسال مسبقاً</t>
+          <t>كم وصلت وكم فُتحت وكم ردّوا</t>
         </is>
       </c>
       <c r="D50" s="18" t="inlineStr">
@@ -3124,9 +3124,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E50" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="F50" s="19" t="inlineStr">
@@ -3158,12 +3158,12 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>عدد رسائل الحملات شهرياً</t>
+          <t>جدولة الإرسال</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>سقف رسائل الحملات المشمولة — رسوم Meta منفصلة</t>
+          <t>تحدّد وقت الإرسال مسبقاً</t>
         </is>
       </c>
       <c r="D51" s="18" t="inlineStr">
@@ -3171,29 +3171,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E51" s="14" t="inlineStr">
-        <is>
-          <t>1,000</t>
-        </is>
-      </c>
-      <c r="F51" s="14" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="G51" s="14" t="inlineStr">
-        <is>
-          <t>مخصّص</t>
-        </is>
-      </c>
-      <c r="H51" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" s="17" t="inlineStr">
-        <is>
-          <t>❌ غير منفّذ</t>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I51" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -3205,96 +3205,96 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
+          <t>عدد رسائل الحملات شهرياً</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>سقف رسائل الحملات المشمولة — رسوم Meta منفصلة</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>1,000</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>مخصّص</t>
+        </is>
+      </c>
+      <c r="H52" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="17" t="inlineStr">
+        <is>
+          <t>❌ غير منفّذ</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>التسويق والحملات</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
           <t>إرسال تدريجي</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>فترة بين كل رسالة وأخرى لحماية رقمك من الحظر</t>
         </is>
       </c>
-      <c r="D52" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G52" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H52" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I52" s="16" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I53" s="16" t="inlineStr">
         <is>
           <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>الفريق والصلاحيات</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>الفريق والصلاحيات</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>أدوار وصلاحيات</t>
-        </is>
-      </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>تحدّد ما يشوفه وما يعمله كل موظف</t>
-        </is>
-      </c>
-      <c r="D54" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F54" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G54" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H54" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I54" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>ساعات عمل ورد خارج الدوام</t>
+          <t>أدوار وصلاحيات</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>رسالة تلقائية خارج أوقات عملكم</t>
+          <t>تحدّد ما يشوفه وما يعمله كل موظف</t>
         </is>
       </c>
       <c r="D55" s="18" t="inlineStr">
@@ -3353,12 +3353,12 @@
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>حالة متاح ومشغول</t>
+          <t>ساعات عمل ورد خارج الدوام</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>الموظف يعلن حالته فلا تصله محادثات وهو مشغول</t>
+          <t>رسالة تلقائية خارج أوقات عملكم</t>
         </is>
       </c>
       <c r="D56" s="18" t="inlineStr">
@@ -3381,9 +3381,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H56" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H56" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I56" s="21" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>هدف زمن الاستجابة لكل قسم</t>
+          <t>حالة متاح ومشغول</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>تحدّد خلال كم دقيقة يجب أن يصل أول رد</t>
+          <t>الموظف يعلن حالته فلا تصله محادثات وهو مشغول</t>
         </is>
       </c>
       <c r="D57" s="18" t="inlineStr">
@@ -3413,9 +3413,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
@@ -3433,9 +3433,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I57" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="I57" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -3447,12 +3447,12 @@
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t>توزيع بكلمة مفتاحية</t>
+          <t>هدف زمن الاستجابة لكل قسم</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>محادثة فيها كلمة «فاتورة» تروح لقسم المحاسبة</t>
+          <t>تحدّد خلال كم دقيقة يجب أن يصل أول رد</t>
         </is>
       </c>
       <c r="D58" s="18" t="inlineStr">
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>سجلّ إجراءات الموظفين</t>
+          <t>توزيع بكلمة مفتاحية</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>تشوف من فتح ومن ردّ ومن أغلق</t>
+          <t>محادثة فيها كلمة «فاتورة» تروح لقسم المحاسبة</t>
         </is>
       </c>
       <c r="D59" s="18" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>توزيع تلقائي متوازن</t>
+          <t>سجلّ إجراءات الموظفين</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>المحادثات تتوزّع على الفريق بالتساوي</t>
+          <t>تشوف من فتح ومن ردّ ومن أغلق</t>
         </is>
       </c>
       <c r="D60" s="18" t="inlineStr">
@@ -3554,9 +3554,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E60" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
@@ -3574,9 +3574,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I60" s="17" t="inlineStr">
-        <is>
-          <t>❌ غير منفّذ</t>
+      <c r="I60" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -3588,96 +3588,96 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
+          <t>توزيع تلقائي متوازن</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>المحادثات تتوزّع على الفريق بالتساوي</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H61" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I61" s="17" t="inlineStr">
+        <is>
+          <t>❌ غير منفّذ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="26" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>الفريق والصلاحيات</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
           <t>التحقق بخطوتين</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>طبقة حماية ثانية على حسابات فريقك</t>
         </is>
       </c>
-      <c r="D61" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F61" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H61" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I61" s="16" t="inlineStr">
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H62" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="16" t="inlineStr">
         <is>
           <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="11" t="inlineStr">
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>العملاء</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>العملاء</t>
-        </is>
-      </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>ملف العميل</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>كل بيانات العميل وسجل محادثاته في مكان واحد</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E63" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F63" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H63" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>تصنيف العملاء</t>
+          <t>ملف العميل</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>تقسم عملاءك لفئات تتعامل مع كل فئة بطريقة</t>
+          <t>كل بيانات العميل وسجل محادثاته في مكان واحد</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
@@ -3736,12 +3736,12 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t>قاعدة المعرفة</t>
+          <t>تصنيف العملاء</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>مقالات وأسئلة شائعة يستخدمها فريقك والمساعد</t>
+          <t>تقسم عملاءك لفئات تتعامل مع كل فئة بطريقة</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -3783,17 +3783,17 @@
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>تقييمات العملاء</t>
+          <t>قاعدة المعرفة</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>يقيّم العميل الخدمة بعد إغلاق المحادثة</t>
-        </is>
-      </c>
-      <c r="D66" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>مقالات وأسئلة شائعة يستخدمها فريقك والمساعد</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
@@ -3811,9 +3811,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H66" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
+      <c r="H66" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I66" s="21" t="inlineStr">
@@ -3830,12 +3830,12 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>الشكاوى والاقتراحات</t>
+          <t>تقييمات العملاء</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>صندوق منفصل للشكاوى تتابعه حتى الإغلاق</t>
+          <t>يقيّم العميل الخدمة بعد إغلاق المحادثة</t>
         </is>
       </c>
       <c r="D67" s="18" t="inlineStr">
@@ -3858,9 +3858,9 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="H67" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H67" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I67" s="21" t="inlineStr">
@@ -3877,96 +3877,96 @@
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
+          <t>الشكاوى والاقتراحات</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>صندوق منفصل للشكاوى تتابعه حتى الإغلاق</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G68" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H68" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="26" customHeight="1">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>العملاء</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
           <t>سجل نشاط العميل</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>كل ما عمله العميل معك بالترتيب الزمني</t>
         </is>
       </c>
-      <c r="D68" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H68" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I68" s="21" t="inlineStr">
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F69" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G69" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H69" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="11" t="inlineStr">
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>التقارير</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="26" customHeight="1">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>التقارير</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>تقارير الأداء</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>لوحة تشوف فيها حجم العمل وأداء الفريق</t>
-        </is>
-      </c>
-      <c r="D70" s="14" t="inlineStr">
-        <is>
-          <t>أساسية</t>
-        </is>
-      </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
-        </is>
-      </c>
-      <c r="F70" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
-        </is>
-      </c>
-      <c r="G70" s="14" t="inlineStr">
-        <is>
-          <t>متقدّمة</t>
-        </is>
-      </c>
-      <c r="H70" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I70" s="21" t="inlineStr">
-        <is>
-          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -3978,37 +3978,37 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>متوسط زمن أول رد</t>
+          <t>تقارير الأداء</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>كم يستنى عميلك قبل أول رد</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="E71" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="F71" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G71" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H71" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>لوحة تشوف فيها حجم العمل وأداء الفريق</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>أساسية</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="G71" s="14" t="inlineStr">
+        <is>
+          <t>متقدّمة</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="I71" s="21" t="inlineStr">
@@ -4025,17 +4025,17 @@
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>ساعات الذروة</t>
+          <t>متوسط زمن أول رد</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>أي ساعات اليوم أكثر ضغطاً لتوزّع فريقك عليها</t>
-        </is>
-      </c>
-      <c r="D72" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>كم يستنى عميلك قبل أول رد</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -4072,12 +4072,12 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>تنبيه عند تأخّر الرد</t>
+          <t>ساعات الذروة</t>
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
-          <t>ينبّهك لما تتجاوز محادثة الوقت المسموح</t>
+          <t>أي ساعات اليوم أكثر ضغطاً لتوزّع فريقك عليها</t>
         </is>
       </c>
       <c r="D73" s="18" t="inlineStr">
@@ -4085,9 +4085,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E73" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E73" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
       <c r="F73" s="19" t="inlineStr">
@@ -4105,9 +4105,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I73" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="I73" s="21" t="inlineStr">
+        <is>
+          <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
@@ -4119,96 +4119,96 @@
       </c>
       <c r="B74" s="12" t="inlineStr">
         <is>
+          <t>تنبيه عند تأخّر الرد</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>ينبّهك لما تتجاوز محادثة الوقت المسموح</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H74" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>التقارير</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
           <t>تصدير التقارير</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
         <is>
           <t>تنزّل تقاريرك ملف CSV</t>
         </is>
       </c>
-      <c r="D74" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F74" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G74" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H74" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I74" s="21" t="inlineStr">
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F75" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G75" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I75" s="21" t="inlineStr">
         <is>
           <t>✅ منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="22" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="11" t="inlineStr">
         <is>
           <t>الربط والدعم</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>الربط والدعم</t>
-        </is>
-      </c>
-      <c r="B76" s="12" t="inlineStr">
-        <is>
-          <t>تكامل API</t>
-        </is>
-      </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>تربط Qhub بأنظمتك الأخرى</t>
-        </is>
-      </c>
-      <c r="D76" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F76" s="14" t="inlineStr">
-        <is>
-          <t>محدود</t>
-        </is>
-      </c>
-      <c r="G76" s="14" t="inlineStr">
-        <is>
-          <t>كامل</t>
-        </is>
-      </c>
-      <c r="H76" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I76" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
         </is>
       </c>
     </row>
@@ -4220,32 +4220,32 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>الدعم</t>
+          <t>تكامل API</t>
         </is>
       </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
-          <t>كيف تتواصل معنا لما تحتاج مساعدة</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>بريد إلكتروني</t>
-        </is>
-      </c>
-      <c r="E77" s="14" t="inlineStr">
-        <is>
-          <t>أولوية</t>
+          <t>تربط Qhub بأنظمتك الأخرى</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F77" s="14" t="inlineStr">
         <is>
-          <t>أولوية</t>
+          <t>محدود</t>
         </is>
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
-          <t>مدير حساب</t>
+          <t>كامل</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -4267,98 +4267,145 @@
       </c>
       <c r="B78" s="12" t="inlineStr">
         <is>
+          <t>الدعم</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>كيف تتواصل معنا لما تحتاج مساعدة</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>بريد إلكتروني</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>أولوية</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>أولوية</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="inlineStr">
+        <is>
+          <t>مدير حساب</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I78" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="26" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>الربط والدعم</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
           <t>اتفاقية مستوى خدمة (SLA)</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C79" s="13" t="inlineStr">
         <is>
           <t>التزام تعاقدي بزمن الرد ونسبة التشغيل</t>
         </is>
       </c>
-      <c r="D78" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E78" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G78" s="19" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="I78" s="17" t="inlineStr">
+      <c r="D79" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="19" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I79" s="17" t="inlineStr">
         <is>
           <t>❌ غير منفّذ</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="30" customHeight="1">
-      <c r="A79" s="3" t="inlineStr">
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>المشمول في كل باقة</t>
         </is>
       </c>
-      <c r="C79" s="3">
-        <f>COUNTIF(H5:H78,"✔")&amp;" صفاً تظهر على الموقع"</f>
+      <c r="C80" s="3">
+        <f>COUNTIF(H5:H79,"✔")&amp;" صفاً تظهر على الموقع"</f>
         <v/>
       </c>
-      <c r="D79" s="3">
-        <f>COUNTIF(D5:D78,"✔")</f>
+      <c r="D80" s="3">
+        <f>COUNTIF(D5:D79,"✔")</f>
         <v/>
       </c>
-      <c r="E79" s="3">
-        <f>COUNTIF(E5:E78,"✔")</f>
+      <c r="E80" s="3">
+        <f>COUNTIF(E5:E79,"✔")</f>
         <v/>
       </c>
-      <c r="F79" s="3">
-        <f>COUNTIF(F5:F78,"✔")</f>
+      <c r="F80" s="3">
+        <f>COUNTIF(F5:F79,"✔")</f>
         <v/>
       </c>
-      <c r="G79" s="3">
-        <f>COUNTIF(G5:G78,"✔")</f>
+      <c r="G80" s="3">
+        <f>COUNTIF(G5:G79,"✔")</f>
         <v/>
       </c>
-      <c r="H79" s="3">
-        <f>COUNTIF(H5:H78,"✔")</f>
+      <c r="H80" s="3">
+        <f>COUNTIF(H5:H79,"✔")</f>
         <v/>
       </c>
-      <c r="I79" s="3">
-        <f>COUNTIF(I5:I78,"✅ منفّذ")&amp;" / "&amp;COUNTIF(I5:I78,"⚠️ جزئي")&amp;" / "&amp;COUNTIF(I5:I78,"❌ غير منفّذ")</f>
+      <c r="I80" s="3">
+        <f>COUNTIF(I5:I79,"✅ منفّذ")&amp;" / "&amp;COUNTIF(I5:I79,"⚠️ جزئي")&amp;" / "&amp;COUNTIF(I5:I79,"❌ غير منفّذ")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A63:I63"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A75:I75"/>
-    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A76:I76"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A70:I70"/>
     <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A69:I69"/>
     <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A62:I62"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4762,7 +4809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5078,12 +5125,32 @@
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>الرسائل الصوتية · تعديل الرسالة خلال 30 دقيقة · فهرسة دورات المحادثة · حالة متاح ومشغول · تصدير التقارير.</t>
+          <t>تطبيق الموظفين على الجوال (منشور على qhub-employee) · الرسائل الصوتية · تعديل الرسالة خلال 30 دقيقة · فهرسة دورات المحادثة · حالة متاح ومشغول · تصدير التقارير.</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>أُضيفت للمصفوفة. يستحق بعضها الظهور على الموقع — قرار تسويقي.</t>
+          <t>أُضيفت للمصفوفة. التطبيق أهمها: مبني ومنشور ولا ذكر له على صفحة الأسعار، بينما respond.io تعرضه على كل باقاتها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>ملاحظة على نطاق هذا التدقيق</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>التدقيق قرأ ريبو اللوحة (chatly) وريبو الموقع (qhub-landing). تطبيق الموظفين في ريبو ثالث، فغاب عن أول نسختين من هذا الملف حتى نُبِّهتُ إليه.</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>إن كانت هناك ريبوهات أخرى في المنتج — لوحة أدمن منفصلة، أو باكند — فقد تحمل مزايا مصنّفة هنا «غير منفّذة».</t>
         </is>
       </c>
     </row>
@@ -5520,14 +5587,14 @@
           <t>تطبيق على كل الباقات بما فيها Starter</t>
         </is>
       </c>
-      <c r="D18" s="30" t="inlineStr">
-        <is>
-          <t>غير موجود</t>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>تطبيق موظفين مبني ومنشور على qhub-employee</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>معروض في ملفك على ثلاث باقات ولا أثر له — إما يُبنى أو يُشطب.</t>
+          <t>موجود عندنا وغير معروض على صفحة الأسعار — فرصة ضائعة. respond.io تعرضه على كل باقة بما فيها الأرخص.</t>
         </is>
       </c>
     </row>

</xml_diff>